<commit_message>
Tighten debt ratio thresholds to 10% healthy and 20% attention
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016z5p4ukvRviThdRJdxEDmy
</commit_message>
<xml_diff>
--- a/biblioteca/materiais/Mini-Sistema-Financeiro-FQC.xlsx
+++ b/biblioteca/materiais/Mini-Sistema-Financeiro-FQC.xlsx
@@ -161,7 +161,7 @@
     <t xml:space="preserve">Executar com controle</t>
   </si>
   <si>
-    <t xml:space="preserve">Referências da Manada: poupança 10%+, endividamento até 30%, reserva de 3 a 6 meses, custo fixo até 50%.</t>
+    <t xml:space="preserve">Referências da Manada: poupança 10%+, endividamento até 10% (atenção até 20%), reserva de 3 a 6 meses, custo fixo até 50%.</t>
   </si>
   <si>
     <t xml:space="preserve">Postergar</t>
@@ -1147,11 +1147,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="4025085"/>
-        <c:axId val="34454580"/>
+        <c:axId val="85585524"/>
+        <c:axId val="90776845"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="4025085"/>
+        <c:axId val="85585524"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1183,7 +1183,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34454580"/>
+        <c:crossAx val="90776845"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1191,7 +1191,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34454580"/>
+        <c:axId val="90776845"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1233,7 +1233,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4025085"/>
+        <c:crossAx val="85585524"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1824,8 +1824,8 @@
         <v>0.105747126436782</v>
       </c>
       <c r="D16" s="20" t="str">
-        <f aca="false">IF(C16&lt;=0.3,"Saudável",IF(C16&lt;=0.4,"Atenção","Alerta"))</f>
-        <v>Saudável</v>
+        <f aca="false">IF(C16&lt;=0.1,"Saudável",IF(C16&lt;=0.2,"Atenção","Alerta"))</f>
+        <v>Atenção</v>
       </c>
       <c r="G16" s="16" t="s">
         <v>40</v>
@@ -2271,7 +2271,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{19E2874B-3666-41FC-B659-40D9738490A1}</x14:id>
+          <x14:id>{226EE1FE-A363-4617-83D9-C57BF1D1BF78}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2299,7 +2299,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{19E2874B-3666-41FC-B659-40D9738490A1}">
+          <x14:cfRule type="dataBar" id="{226EE1FE-A363-4617-83D9-C57BF1D1BF78}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -22229,7 +22229,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3C2F2B42-18B6-4D21-B434-56949F5D3FA8}</x14:id>
+          <x14:id>{D8D9D82F-DD7B-4F4A-BDC3-D471CF1024D1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22245,7 +22245,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3C2F2B42-18B6-4D21-B434-56949F5D3FA8}">
+          <x14:cfRule type="dataBar" id="{D8D9D82F-DD7B-4F4A-BDC3-D471CF1024D1}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>